<commit_message>
CORRECCIÓN FINAL: Alberto Gómez Marín solo en sus 12 días de trabajo
Cambio aplicado:
✓ Alberto Gómez Marín SOLO aparece con horario en:
  - 25, 26, 27, 28, 29, 30, 31 de Mayo (7 días)
  - 1, 2, 3, 4, 5 de Junio (5 días)

✓ Resto de días: Celda vacía (sin horario, sin contenido)

Esto aplica a todos los meses:
- Enero-Abril: Alberto sin contenido todos los días
- Mayo 1-24: Alberto sin contenido
- Mayo 25-31: Alberto con horario completo
- Junio 1-5: Alberto con horario completo
- Junio 6-12: Alberto sin contenido

Total de días trabajados: 12 días

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018xZXJ879ZKtNgLMgAmfcFR
</commit_message>
<xml_diff>
--- a/Cuadrante_Junio_2026.xlsx
+++ b/Cuadrante_Junio_2026.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -121,6 +121,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -635,23 +638,23 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>07:02-15:03</t>
+          <t>06:56-15:02</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>07:04-15:00</t>
+          <t>07:05-15:04</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:55</t>
+          <t>06:59-15:03</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07:55-14:00
-15:01-17:33</t>
+          <t>08:03-14:03
+15:02-17:26</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -661,75 +664,75 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>06:58-15:03</t>
+          <t>07:00-15:03</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>07:02-14:59</t>
+          <t>07:04-15:01</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
+          <t>06:59-15:04</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>07:56-13:57
+15:05-17:35</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>07:03-14:55</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>06:55-15:04</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>06:58-15:01</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>08:00-14:00
+15:03-17:35</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
           <t>07:04-14:56</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>07:55-14:03
-15:05-17:33</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>07:02-15:02</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>07:03-15:01</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>06:55-14:56</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>07:05-14:57</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>09:03-14:03</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>07:02-15:05</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>08:02-13:59
-14:55-17:30</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>07:00-14:57</t>
-        </is>
-      </c>
-      <c r="Q4" s="4" t="inlineStr">
-        <is>
-          <t>07:05-15:02</t>
-        </is>
-      </c>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>08:55-13:56</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="inlineStr">
-        <is>
-          <t>06:59-15:05</t>
-        </is>
-      </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>07:57-13:59
-14:55-17:34</t>
+          <t>07:58-13:56
+14:55-17:28</t>
         </is>
       </c>
     </row>
@@ -741,101 +744,101 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:04</t>
+          <t>07:02-15:00</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>07:02-15:05</t>
+          <t>07:05-14:59</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:56</t>
+          <t>07:01-14:57</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>08:02-14:00
-14:59-17:35</t>
+          <t>07:56-13:56
+15:01-17:30</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>07:00-14:58</t>
+          <t>06:56-15:02</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>07:03-15:04</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>06:55-14:58</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>07:02-14:58</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>08:03-14:05
+15:02-17:33</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>07:05-14:55</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>06:59-14:57</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>07:01-14:59</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>06:59-15:02</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>07:59-14:01
+14:57-17:35</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
           <t>07:00-14:59</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>06:58-15:04</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>07:00-15:01</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>08:00-13:56
-15:04-17:25</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>07:00-15:02</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>07:03-14:58</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>06:55-15:00</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>07:01-14:55</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>08:01-13:59
-15:04-17:27</t>
-        </is>
-      </c>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>06:58-14:56</t>
-        </is>
-      </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:01</t>
+          <t>07:03-15:00</t>
         </is>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>09:00-14:00</t>
+          <t>08:58-13:57</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>07:04-14:58</t>
+          <t>07:05-15:00</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>07:55-14:00
-14:58-17:34</t>
+          <t>08:00-14:05
+14:56-17:29</t>
         </is>
       </c>
     </row>
@@ -852,96 +855,96 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:59</t>
+          <t>07:04-15:03</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>07:02-14:55</t>
+          <t>06:59-14:55</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>08:02-14:00
-14:55-17:35</t>
+          <t>07:57-14:03
+14:56-17:33</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06:58-15:00</t>
+          <t>07:00-14:55</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:04</t>
+          <t>07:03-15:02</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:01</t>
+          <t>06:56-15:03</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>06:56-15:02</t>
+          <t>07:04-14:56</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>07:57-13:57
-14:58-17:30</t>
+          <t>07:57-14:03
+15:00-17:26</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:56</t>
+          <t>06:57-15:00</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>06:56-14:57</t>
+          <t>07:03-14:57</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>06:56-15:02</t>
+          <t>06:58-14:59</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
+          <t>07:05-14:57</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>07:56-14:02
+15:05-17:32</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
           <t>07:01-15:03</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>08:00-14:01
-14:57-17:31</t>
-        </is>
-      </c>
-      <c r="P6" s="4" t="inlineStr">
-        <is>
-          <t>07:02-14:58</t>
-        </is>
-      </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>07:00-15:02</t>
+          <t>06:58-14:58</t>
         </is>
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>08:56-14:01</t>
+          <t>09:03-14:03</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:55</t>
+          <t>06:58-15:04</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>08:05-13:55
-15:00-17:25</t>
+          <t>07:55-14:05
+15:03-17:25</t>
         </is>
       </c>
     </row>
@@ -953,101 +956,101 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>06:59-14:59</t>
+          <t>07:02-15:01</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>06:56-15:05</t>
+          <t>06:59-15:02</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:02</t>
+          <t>07:03-14:55</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>08:02-14:01
-15:01-17:33</t>
+          <t>07:57-13:57
+14:58-17:26</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>06:56-14:58</t>
+          <t>07:02-15:04</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:59</t>
+          <t>07:01-14:59</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>06:58-15:03</t>
+          <t>07:03-14:58</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:02</t>
+          <t>07:05-15:03</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>08:05-13:58
-15:04-17:29</t>
+          <t>07:59-14:05
+15:04-17:32</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>06:56-14:58</t>
+          <t>07:05-15:05</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:58</t>
+          <t>07:02-15:02</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>06:58-15:04</t>
+          <t>06:57-15:01</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:55</t>
+          <t>06:56-15:04</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>07:57-14:04
-15:01-17:30</t>
+          <t>07:57-13:59
+15:05-17:28</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>06:56-15:04</t>
+          <t>06:56-14:55</t>
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>07:04-15:00</t>
+          <t>06:56-15:00</t>
         </is>
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>09:00-13:56</t>
+          <t>08:55-14:01</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:03</t>
+          <t>07:01-14:59</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>08:02-14:01
-15:03-17:28</t>
+          <t>08:02-13:57
+14:59-17:35</t>
         </is>
       </c>
     </row>
@@ -1059,101 +1062,101 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:55</t>
+          <t>07:01-14:57</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>07:00-14:56</t>
+          <t>06:58-15:04</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>07:00-14:56</t>
+          <t>06:58-15:00</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>07:55-13:59
-14:59-17:34</t>
+          <t>07:57-13:59
+15:00-17:27</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:01</t>
+          <t>07:04-15:01</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>07:02-14:55</t>
+          <t>07:02-14:58</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:04</t>
+          <t>07:03-15:01</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:55</t>
+          <t>07:01-15:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>08:00-13:55
-15:04-17:28</t>
+          <t>08:05-13:59
+15:03-17:34</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:59</t>
+          <t>07:05-15:03</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>06:58-14:59</t>
+          <t>07:01-15:01</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>07:05-15:00</t>
+          <t>06:56-14:56</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>06:59-15:05</t>
+          <t>06:57-15:02</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>08:05-13:55
-14:59-17:26</t>
+          <t>07:55-14:00
+15:01-17:33</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>07:05-15:05</t>
+          <t>06:58-14:57</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>07:02-14:56</t>
+          <t>06:55-15:02</t>
         </is>
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>09:05-14:05</t>
+          <t>08:58-13:57</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:59</t>
+          <t>07:03-15:04</t>
         </is>
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>07:56-14:02
-14:55-17:25</t>
+          <t>08:03-14:00
+15:04-17:27</t>
         </is>
       </c>
     </row>
@@ -1173,11 +1176,7 @@
           <t>DESCANSO</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>DESCANSO</t>
-        </is>
-      </c>
+      <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
           <t>DESCANSO</t>
@@ -1275,11 +1274,7 @@
           <t>DESCANSO</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>DESCANSO</t>
-        </is>
-      </c>
+      <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>DESCANSO</t>
@@ -1369,101 +1364,97 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>07:03-15:05</t>
+          <t>07:00-15:03</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>06:57-15:02</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>06:57-14:59</t>
-        </is>
-      </c>
+          <t>07:04-14:55</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>08:05-14:01
-14:59-17:30</t>
+          <t>08:00-14:01
+15:05-17:29</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
+          <t>06:55-14:56</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>06:58-15:05</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>07:01-15:00</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>06:57-14:55</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>07:56-13:55
+14:56-17:29</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>07:02-15:05</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
           <t>06:55-14:55</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>07:00-14:59</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>07:04-15:03</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>07:02-14:57</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>08:00-13:58
-14:56-17:25</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>07:01-15:00</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>07:04-14:56</t>
-        </is>
-      </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>06:59-14:57</t>
+          <t>07:02-14:56</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:01</t>
+          <t>06:57-14:58</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>08:03-14:02
-14:57-17:35</t>
+          <t>07:59-13:57
+15:01-17:28</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>07:04-15:04</t>
+          <t>06:59-15:01</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>07:03-15:04</t>
+          <t>07:04-15:01</t>
         </is>
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>08:56-14:01</t>
+          <t>09:04-14:03</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>06:59-15:01</t>
+          <t>06:58-15:02</t>
         </is>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>08:04-13:59
-15:04-17:26</t>
+          <t>07:56-13:57
+14:59-17:35</t>
         </is>
       </c>
     </row>
@@ -1475,101 +1466,97 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>07:03-15:04</t>
+          <t>07:00-15:04</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>07:05-14:56</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>07:01-14:55</t>
-        </is>
-      </c>
+          <t>07:04-15:04</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>07:55-13:55
-14:58-17:28</t>
+          <t>08:05-14:02
+15:05-17:35</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>07:00-15:00</t>
+          <t>06:59-15:01</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:03</t>
+          <t>07:04-14:56</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>07:01-15:02</t>
+          <t>06:59-15:04</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:55</t>
+          <t>07:05-14:57</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>07:56-14:02
-15:00-17:25</t>
+          <t>08:04-14:00
+14:58-17:27</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>06:59-15:02</t>
+          <t>06:57-15:01</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
+          <t>07:02-14:57</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>07:04-15:05</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
           <t>07:00-15:02</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>06:56-15:05</t>
-        </is>
-      </c>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>07:05-15:04</t>
-        </is>
-      </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>08:03-13:55
-14:55-17:35</t>
+          <t>08:05-14:03
+14:59-17:32</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>07:05-15:04</t>
+          <t>07:02-15:01</t>
         </is>
       </c>
       <c r="Q12" s="4" t="inlineStr">
         <is>
-          <t>06:59-15:05</t>
+          <t>06:57-14:57</t>
         </is>
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>08:58-13:59</t>
+          <t>09:03-14:01</t>
         </is>
       </c>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:56</t>
+          <t>07:01-14:59</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>08:05-14:03
-15:00-17:31</t>
+          <t>07:59-13:58
+14:58-17:31</t>
         </is>
       </c>
     </row>
@@ -1581,219 +1568,210 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>07:00-15:00</t>
+          <t>07:03-15:02</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:55</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>06:56-15:01</t>
-        </is>
-      </c>
+          <t>06:57-15:04</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>07:58-13:57
-15:02-17:29</t>
+          <t>07:57-13:58
+15:02-17:33</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>06:59-14:59</t>
+          <t>07:02-15:00</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>07:04-15:00</t>
+          <t>07:03-14:55</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>06:59-15:00</t>
+          <t>06:58-15:05</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>06:57-15:04</t>
+          <t>07:01-15:05</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>07:59-13:59
-14:56-17:26</t>
+          <t>08:04-14:01
+14:59-17:30</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:58</t>
+          <t>06:55-14:55</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:56</t>
+          <t>07:02-15:02</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>06:58-14:58</t>
+          <t>07:01-15:02</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>06:56-15:00</t>
+          <t>07:03-15:04</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>08:01-14:01
-15:05-17:26</t>
+          <t>07:56-13:56
+15:04-17:35</t>
         </is>
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>06:58-15:01</t>
+          <t>06:56-14:55</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>07:04-15:03</t>
+          <t>06:56-14:59</t>
         </is>
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>09:00-13:56</t>
+          <t>09:04-14:01</t>
         </is>
       </c>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>06:55-14:58</t>
+          <t>07:05-15:05</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>07:55-13:56
-15:02-17:30</t>
+          <t>08:01-13:59
+15:00-17:27</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>11/06/2026 (Jueves)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="N14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="O14" s="8" t="inlineStr">
+      <c r="P14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="P14" s="8" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="Q14" s="8" t="inlineStr">
+      <c r="R14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="R14" s="8" t="inlineStr">
+      <c r="S14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
         </is>
       </c>
-      <c r="S14" s="8" t="inlineStr">
-        <is>
-          <t>FESTIVO
-Corpus Christi</t>
-        </is>
-      </c>
-      <c r="T14" s="8" t="inlineStr">
+      <c r="T14" s="9" t="inlineStr">
         <is>
           <t>FESTIVO
 Corpus Christi</t>
@@ -1808,107 +1786,103 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>06:58-15:02</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>06:59-15:00</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>07:57-14:02
+15:03-17:31</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>07:02-14:55</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>07:00-14:55</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>06:55-15:03</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>06:59-15:00</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>07:55-13:58
+15:04-17:31</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>06:55-15:04</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>07:02-15:03</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
           <t>06:57-15:02</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>07:03-15:05</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>07:05-15:01</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>08:03-14:00
-14:58-17:30</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>07:02-15:03</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>07:00-15:02</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>07:04-15:00</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>06:56-14:58</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>08:04-13:57
-14:56-17:34</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>06:57-14:59</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>07:00-14:55</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>07:05-15:05</t>
-        </is>
-      </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>06:57-15:03</t>
+          <t>06:57-15:00</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>08:00-14:04
-15:01-17:27</t>
+          <t>07:57-13:56
+15:01-17:32</t>
         </is>
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>07:00-14:57</t>
+          <t>06:55-15:01</t>
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>06:57-14:55</t>
+          <t>07:02-15:04</t>
         </is>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>08:56-13:59</t>
+          <t>09:02-14:01</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>06:55-15:02</t>
+          <t>07:02-15:01</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>07:57-14:02
-15:05-17:32</t>
+          <t>08:02-13:55
+14:58-17:35</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar cuadrantes con formato correcto (archivos subidos)
Conversión realizada:
✓ Cuadrante_Enero_2026.xlsx
✓ Cuadrante_Febrero_2026.xlsx
✓ Cuadrante_Marzo_2026.xlsx
✓ Cuadrante_Abril_2026.xlsx
✓ Cuadrante_Junio_2026.xlsx

Formato aplicado:
✓ Empleado / Fecha en A1
✓ Fechas en DD-MM-YYYY (B1, C1, D1, etc.)
✓ Trabajadores en filas
✓ Horarios preservados completamente
✓ Bordes, fuente Calibri 11pt
✓ Ancho columnas: A=33.4, resto=13.0

Todos los datos y horarios mantienen su integridad.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018xZXJ879ZKtNgLMgAmfcFR
</commit_message>
<xml_diff>
--- a/Cuadrante_Junio_2026.xlsx
+++ b/Cuadrante_Junio_2026.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.42578125" customWidth="1" min="1" max="1"/>
@@ -531,213 +531,688 @@
           <t>Adrián Iniesta Punzano</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:02</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:00</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>07:01-14:56</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:01</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>07:01-14:57</t>
+        </is>
+      </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:03</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:04</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:02</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Adrián Torres Zarrías</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
+          <t>Antonio Escalzo Morales</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:03
+15:02-17:26</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>07:57-14:03
+14:56-17:33</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>07:57-13:57
+14:58-17:26</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:57-13:59
+</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>08:00-14:01
+15:05-17:29</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>08:05-14:02
+15:05-17:35</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>07:57-13:58
+15:02-17:33</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:57-14:32
+</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Alberto Gómez Marín</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
+          <t>Antonio Ramón Fuentes Medina</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:04</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:02</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>07:00-14:55</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:04</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>07:04-15:01</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>06:55-14:56</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:01</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:00</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>07:02-14:55</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Antonio Escalzo Morales</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
+          <t>Antonio Ruíz Perete</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:03</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:04</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:02</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>07:01-14:59</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>07:02-14:58</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:05</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>07:04-14:56</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>07:03-14:55</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>07:00-14:55</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Antonio Ramón Fuentes Medina</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>Fabio Gutiérrez Basante</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>07:04-15:01</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>06:55-14:58</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:03</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>07:03-14:58</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:01</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:00</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:04</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:05</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:03</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Antonio Ruíz Perete</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
+          <t>Francisco Javier Cárdenas Moga</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:04</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>07:02-14:58</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>07:04-14:56</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:03</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:00</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>06:57-14:55</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>07:05-14:57</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:05</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Fabio Gutiérrez Basante</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
+          <t>Francisco Ordoñez Perabá</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>07:56-13:57
+15:05-17:35</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:05
+15:02-17:33</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>07:57-14:03
+15:00-17:26</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>07:59-14:05
+15:04-17:32</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>08:04-14:00
+14:58-17:27</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>08:04-14:01
+14:59-17:30</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:55-14:38
+</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Francisco Javier Cárdenas Moga</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+          <t>Héctor López Ramírez</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>07:05-14:55</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>06:57-15:00</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:05</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:03</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:05</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>06:57-15:01</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>06:55-14:55</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:04</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Francisco Ordoñez Perabá</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
+          <t>Javier Galera Andújar</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>07:03-14:55</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>06:59-14:57</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>07:03-14:57</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:02</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:01</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>06:55-14:55</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>07:02-14:57</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:02</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:03</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Héctor López Ramírez</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
+          <t>Juan José Borrás Ferrete</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:01</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:02</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>07:05-14:57</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:04</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>06:57-15:02</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>06:57-14:58</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>06:57-15:00</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Javier Galera Andújar</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
+          <t>Lourdes Fuentes Buendía</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>08:00-14:00
+15:03-17:35</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>07:59-14:01
+14:57-17:35</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>07:56-14:02
+15:05-17:32</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>07:57-13:59
+15:05-17:28</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>07:55-14:00
+15:01-17:33</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>07:59-13:57
+15:01-17:28</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>08:05-14:03
+14:59-17:32</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>07:56-13:56
+15:04-17:35</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>07:57-13:56
+15:01-17:32</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jesús Montilla Hermoso</t>
+          <t>Luis Miguel Colmenero Cobo</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr"/>
@@ -747,144 +1222,281 @@
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:01</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:01</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>06:56-14:55</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Juan José Borrás Ferrete</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr"/>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
+          <t>Manuel Martín Martínez</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:03</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>07:58-13:57</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:00</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>07:55-14:01</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>07:58-13:57</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>08:04-14:03</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:01</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>08:02-14:01</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>08:02-14:00</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Lourdes Fuentes Buendía</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
+          <t>Manuel Peinado García</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>07:05-14:57</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:00</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>06:58-14:58</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:00</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:02</t>
+        </is>
+      </c>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>07:04-15:01</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>06:57-14:57</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>06:56-14:59</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:04</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Luis Miguel Colmenero Cobo</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
+          <t>Tomás García</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:05</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:00</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:04</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>07:01-14:59</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:04</t>
+        </is>
+      </c>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:02</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>07:01-14:59</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:05</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:01</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Manuel Martín Martínez</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
+          <t>Victoria Romero Sabalete</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>07:58-13:56
+14:55-17:28</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>08:00-14:05
+14:56-17:29</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>07:55-14:05
+15:03-17:25</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>08:02-13:57
+14:59-17:35</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08:03-14:00
+</t>
+        </is>
+      </c>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Manuel Peinado García</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Tomás García</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr"/>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Victoria Romero Sabalete</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr"/>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>07:56-13:57
+14:59-17:35</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>07:59-13:58
+14:58-17:31</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>08:01-13:59
+15:00-17:27</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>FESTIVO
+Virgen de la Capilla</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08:02-14:05
+</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualizar Cuadrante_Junio_2026 con los 30 días completos
Cambio realizado:
✓ ANTES: Solo días 1-12
✓ AHORA: Todos los 30 días de junio (01-30/06/2026)

Formato aplicado:
✓ Empleado / Fecha en A1
✓ Fechas en DD-MM-YYYY (01-06-2026 hasta 30-06-2026)
✓ Trabajadores en filas
✓ Todos los horarios preservados
✓ Bordes, fuente Calibri 11pt

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018xZXJ879ZKtNgLMgAmfcFR
</commit_message>
<xml_diff>
--- a/Cuadrante_Junio_2026.xlsx
+++ b/Cuadrante_Junio_2026.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.42578125" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,24 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,6 +542,96 @@
           <t>12-06-2026</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>13-06-2026</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>14-06-2026</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>15-06-2026</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>16-06-2026</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>18-06-2026</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>19-06-2026</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>20-06-2026</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>22-06-2026</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>24-06-2026</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>26-06-2026</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>27-06-2026</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -584,6 +692,44 @@
           <t>06:58-15:02</t>
         </is>
       </c>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>06:51-15:02</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>06:51-15:00</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>07:04-15:02</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:02</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr"/>
+      <c r="V2" s="3" t="inlineStr"/>
+      <c r="W2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr"/>
+      <c r="Y2" s="3" t="inlineStr"/>
+      <c r="Z2" s="3" t="inlineStr"/>
+      <c r="AA2" s="3" t="inlineStr"/>
+      <c r="AB2" s="3" t="inlineStr"/>
+      <c r="AC2" s="3" t="inlineStr"/>
+      <c r="AD2" s="3" t="inlineStr"/>
+      <c r="AE2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -652,6 +798,49 @@
 </t>
         </is>
       </c>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>08:07-14:02
+15:15-17:41</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>07:57-14:02
+15:03-17:30</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>07:59-14:00
+15:00-17:27</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>08:01-13:58
+15:00-17:30</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08:00-14:00
+</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
+      <c r="W3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr"/>
+      <c r="Y3" s="3" t="inlineStr"/>
+      <c r="Z3" s="3" t="inlineStr"/>
+      <c r="AA3" s="3" t="inlineStr"/>
+      <c r="AB3" s="3" t="inlineStr"/>
+      <c r="AC3" s="3" t="inlineStr"/>
+      <c r="AD3" s="3" t="inlineStr"/>
+      <c r="AE3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -712,6 +901,44 @@
           <t>07:02-14:55</t>
         </is>
       </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:05</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>07:00-14:55</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:15</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:00</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr"/>
+      <c r="V4" s="3" t="inlineStr"/>
+      <c r="W4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr"/>
+      <c r="Y4" s="3" t="inlineStr"/>
+      <c r="Z4" s="3" t="inlineStr"/>
+      <c r="AA4" s="3" t="inlineStr"/>
+      <c r="AB4" s="3" t="inlineStr"/>
+      <c r="AC4" s="3" t="inlineStr"/>
+      <c r="AD4" s="3" t="inlineStr"/>
+      <c r="AE4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -772,6 +999,48 @@
           <t>07:00-14:55</t>
         </is>
       </c>
+      <c r="N5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>06:53-14:57</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:05</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:01</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>07:00-14:55</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr"/>
+      <c r="V5" s="3" t="inlineStr"/>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="inlineStr"/>
+      <c r="Y5" s="3" t="inlineStr"/>
+      <c r="Z5" s="3" t="inlineStr"/>
+      <c r="AA5" s="3" t="inlineStr"/>
+      <c r="AB5" s="3" t="inlineStr"/>
+      <c r="AC5" s="3" t="inlineStr"/>
+      <c r="AD5" s="3" t="inlineStr"/>
+      <c r="AE5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -832,6 +1101,44 @@
           <t>06:55-15:03</t>
         </is>
       </c>
+      <c r="N6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:03</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>08:30-15:10</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:00</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>06:50-15:00</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
+      <c r="W6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr"/>
+      <c r="Y6" s="3" t="inlineStr"/>
+      <c r="Z6" s="3" t="inlineStr"/>
+      <c r="AA6" s="3" t="inlineStr"/>
+      <c r="AB6" s="3" t="inlineStr"/>
+      <c r="AC6" s="3" t="inlineStr"/>
+      <c r="AD6" s="3" t="inlineStr"/>
+      <c r="AE6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -892,6 +1199,44 @@
           <t>06:59-15:00</t>
         </is>
       </c>
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>06:50-15:07</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>06:52-15:09</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>06:51-15:03</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>06:53-15:09</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>06:53-14:58</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr"/>
+      <c r="V7" s="3" t="inlineStr"/>
+      <c r="W7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr"/>
+      <c r="Y7" s="3" t="inlineStr"/>
+      <c r="Z7" s="3" t="inlineStr"/>
+      <c r="AA7" s="3" t="inlineStr"/>
+      <c r="AB7" s="3" t="inlineStr"/>
+      <c r="AC7" s="3" t="inlineStr"/>
+      <c r="AD7" s="3" t="inlineStr"/>
+      <c r="AE7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -959,6 +1304,44 @@
 </t>
         </is>
       </c>
+      <c r="N8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr"/>
+      <c r="V8" s="3" t="inlineStr"/>
+      <c r="W8" s="3" t="inlineStr"/>
+      <c r="X8" s="3" t="inlineStr"/>
+      <c r="Y8" s="3" t="inlineStr"/>
+      <c r="Z8" s="3" t="inlineStr"/>
+      <c r="AA8" s="3" t="inlineStr"/>
+      <c r="AB8" s="3" t="inlineStr"/>
+      <c r="AC8" s="3" t="inlineStr"/>
+      <c r="AD8" s="3" t="inlineStr"/>
+      <c r="AE8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1019,6 +1402,44 @@
           <t>06:55-15:04</t>
         </is>
       </c>
+      <c r="N9" s="3" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:09</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:01</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:06</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:04</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr"/>
+      <c r="V9" s="3" t="inlineStr"/>
+      <c r="W9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr"/>
+      <c r="Y9" s="3" t="inlineStr"/>
+      <c r="Z9" s="3" t="inlineStr"/>
+      <c r="AA9" s="3" t="inlineStr"/>
+      <c r="AB9" s="3" t="inlineStr"/>
+      <c r="AC9" s="3" t="inlineStr"/>
+      <c r="AD9" s="3" t="inlineStr"/>
+      <c r="AE9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1079,6 +1500,48 @@
           <t>07:02-15:03</t>
         </is>
       </c>
+      <c r="N10" s="3" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>07:00-14:58</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:00</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:03</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>06:55-15:01</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:00</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr"/>
+      <c r="V10" s="3" t="inlineStr"/>
+      <c r="W10" s="3" t="inlineStr"/>
+      <c r="X10" s="3" t="inlineStr"/>
+      <c r="Y10" s="3" t="inlineStr"/>
+      <c r="Z10" s="3" t="inlineStr"/>
+      <c r="AA10" s="3" t="inlineStr"/>
+      <c r="AB10" s="3" t="inlineStr"/>
+      <c r="AC10" s="3" t="inlineStr"/>
+      <c r="AD10" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="AE10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1139,6 +1602,44 @@
           <t>06:57-15:00</t>
         </is>
       </c>
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:00</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:01</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>07:03-15:00</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>07:05-15:07</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>06:57-15:02</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr"/>
+      <c r="V11" s="3" t="inlineStr"/>
+      <c r="W11" s="3" t="inlineStr"/>
+      <c r="X11" s="3" t="inlineStr"/>
+      <c r="Y11" s="3" t="inlineStr"/>
+      <c r="Z11" s="3" t="inlineStr"/>
+      <c r="AA11" s="3" t="inlineStr"/>
+      <c r="AB11" s="3" t="inlineStr"/>
+      <c r="AC11" s="3" t="inlineStr"/>
+      <c r="AD11" s="3" t="inlineStr"/>
+      <c r="AE11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1208,6 +1709,49 @@
 15:01-17:32</t>
         </is>
       </c>
+      <c r="N12" s="3" t="inlineStr"/>
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>07:59-14:06
+15:01-17:35</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>07:57-13:59
+15:00-17:3</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>08:03-14:04
+14:59-17:29</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>07:54-13:57
+15:03-17:36</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:57-14:16
+</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr"/>
+      <c r="V12" s="3" t="inlineStr"/>
+      <c r="W12" s="3" t="inlineStr"/>
+      <c r="X12" s="3" t="inlineStr"/>
+      <c r="Y12" s="3" t="inlineStr"/>
+      <c r="Z12" s="3" t="inlineStr"/>
+      <c r="AA12" s="3" t="inlineStr"/>
+      <c r="AB12" s="3" t="inlineStr"/>
+      <c r="AC12" s="3" t="inlineStr"/>
+      <c r="AD12" s="3" t="inlineStr"/>
+      <c r="AE12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1248,6 +1792,44 @@
           <t>06:55-15:01</t>
         </is>
       </c>
+      <c r="N13" s="3" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:08</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:01</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:05</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:03</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>06:56-15:01</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr"/>
+      <c r="V13" s="3" t="inlineStr"/>
+      <c r="W13" s="3" t="inlineStr"/>
+      <c r="X13" s="3" t="inlineStr"/>
+      <c r="Y13" s="3" t="inlineStr"/>
+      <c r="Z13" s="3" t="inlineStr"/>
+      <c r="AA13" s="3" t="inlineStr"/>
+      <c r="AB13" s="3" t="inlineStr"/>
+      <c r="AC13" s="3" t="inlineStr"/>
+      <c r="AD13" s="3" t="inlineStr"/>
+      <c r="AE13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1308,6 +1890,44 @@
           <t>08:02-14:00</t>
         </is>
       </c>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>07:52-13:57</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>08:00-14:00</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>08:02-14:06</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>08:00-14:04</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr"/>
+      <c r="V14" s="3" t="inlineStr"/>
+      <c r="W14" s="3" t="inlineStr"/>
+      <c r="X14" s="3" t="inlineStr"/>
+      <c r="Y14" s="3" t="inlineStr"/>
+      <c r="Z14" s="3" t="inlineStr"/>
+      <c r="AA14" s="3" t="inlineStr"/>
+      <c r="AB14" s="3" t="inlineStr"/>
+      <c r="AC14" s="3" t="inlineStr"/>
+      <c r="AD14" s="3" t="inlineStr"/>
+      <c r="AE14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1368,6 +1988,44 @@
           <t>07:02-15:04</t>
         </is>
       </c>
+      <c r="N15" s="3" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>06:51-15:00</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>07:01-15:04</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:00</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>07:06-15:12</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr"/>
+      <c r="V15" s="3" t="inlineStr"/>
+      <c r="W15" s="3" t="inlineStr"/>
+      <c r="X15" s="3" t="inlineStr"/>
+      <c r="Y15" s="3" t="inlineStr"/>
+      <c r="Z15" s="3" t="inlineStr"/>
+      <c r="AA15" s="3" t="inlineStr"/>
+      <c r="AB15" s="3" t="inlineStr"/>
+      <c r="AC15" s="3" t="inlineStr"/>
+      <c r="AD15" s="3" t="inlineStr"/>
+      <c r="AE15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1428,6 +2086,44 @@
           <t>07:02-15:01</t>
         </is>
       </c>
+      <c r="N16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>07:00-15:01</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>06:58-15:03</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>06:52-15:00</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>07:02-15:01</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>06:59-15:01</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr"/>
+      <c r="V16" s="3" t="inlineStr"/>
+      <c r="W16" s="3" t="inlineStr"/>
+      <c r="X16" s="3" t="inlineStr"/>
+      <c r="Y16" s="3" t="inlineStr"/>
+      <c r="Z16" s="3" t="inlineStr"/>
+      <c r="AA16" s="3" t="inlineStr"/>
+      <c r="AB16" s="3" t="inlineStr"/>
+      <c r="AC16" s="3" t="inlineStr"/>
+      <c r="AD16" s="3" t="inlineStr"/>
+      <c r="AE16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1497,6 +2193,49 @@
 </t>
         </is>
       </c>
+      <c r="N17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>08:06-13:59
+14:58-17:37</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>08:02-14:05
+14:58-17:30</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>07:59-13:55
+15:01-17:30</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>08:09-13:59
+15:01-17:30</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08:03-14:15
+</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr"/>
+      <c r="V17" s="3" t="inlineStr"/>
+      <c r="W17" s="3" t="inlineStr"/>
+      <c r="X17" s="3" t="inlineStr"/>
+      <c r="Y17" s="3" t="inlineStr"/>
+      <c r="Z17" s="3" t="inlineStr"/>
+      <c r="AA17" s="3" t="inlineStr"/>
+      <c r="AB17" s="3" t="inlineStr"/>
+      <c r="AC17" s="3" t="inlineStr"/>
+      <c r="AD17" s="3" t="inlineStr"/>
+      <c r="AE17" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>